<commit_message>
first monitor, Steklova, Role OSBB Observer, Video Observation
</commit_message>
<xml_diff>
--- a/outputs/2026-09-18-osbb-vehicles/OSBB_Все_автомобили_2026-09-18.xlsx
+++ b/outputs/2026-09-18-osbb-vehicles/OSBB_Все_автомобили_2026-09-18.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/san/Developer/Projects/OSBB_cl/outputs/2026-09-18-osbb-vehicles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9363D431-8750-A648-B5D3-FEAE174088B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13446534-49B2-1F48-98E7-1AD45ADC71B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4377,6 +4377,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>